<commit_message>
Update of docs. Update of URL and fix format of title for test
</commit_message>
<xml_diff>
--- a/docs/TestCases.xlsx
+++ b/docs/TestCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arcigo/Documents/Projects/BigBankDemo/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1722BEF-0336-FD48-B6CD-340DFCFE854F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9ECF041-D743-984B-9C0B-06E90C936E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{5A36BFF6-BC86-D248-B9E6-C6BC71C126C7}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{5A36BFF6-BC86-D248-B9E6-C6BC71C126C7}"/>
   </bookViews>
   <sheets>
     <sheet name="UI (part 1)" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="155">
   <si>
     <t>Test Case</t>
   </si>
@@ -4395,28 +4395,6 @@
   <si>
     <r>
       <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Kuumakse</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> is recalculated every certain amount of time. For this case, the value is approximately €730.02. When the loan quote is finished, the kuumakse may remain as it is or change.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
@@ -4507,6 +4485,114 @@
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If I press the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Enter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> key after filling any of the inputs of the form, or when I use the sliders, the modal closes. Is this an expected behavior? If not, this condition from the assessment is not met: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>«Calculator changes should not be saved until the "Jätka" button is clicked»</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>* Kuumakse</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is recalculated every certain amount of time. For this case, the value is approximately €730.02. When the loan quote is finished, the kuumakse may remain as it is or change.
+* If I press the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Enter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> key after filling any of the inputs of the form, or when I use the sliders, the modal closes. Is this an expected behavior? If not, this condition from the assessment is not met: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>«Calculator changes should not be saved until the "Jätka" button is clicked»</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>.</t>
@@ -4675,9 +4761,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4688,9 +4771,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -4714,7 +4794,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4729,26 +4809,20 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -4757,6 +4831,18 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5105,217 +5191,217 @@
     <col min="7" max="7" width="29.83203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="28.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="10.83203125" style="22"/>
+    <col min="10" max="11" width="10.83203125" style="19"/>
     <col min="12" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
     </row>
     <row r="2" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="J2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="26" t="s">
+      <c r="K2" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="119" x14ac:dyDescent="0.2">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="H3" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J3" s="21" t="s">
+      <c r="J3" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="K3" s="21" t="s">
+      <c r="K3" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="8" t="s">
+      <c r="L3" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="85" x14ac:dyDescent="0.2">
-      <c r="A4" s="21" t="s">
+    <row r="4" spans="1:12" ht="68" x14ac:dyDescent="0.2">
+      <c r="A4" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="21" t="s">
+      <c r="J4" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="K4" s="21" t="s">
+      <c r="K4" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="L4" s="8" t="s">
+      <c r="L4" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="27"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
+      <c r="A5" s="22"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="22"/>
-      <c r="C6" s="19"/>
+      <c r="A6" s="19"/>
+      <c r="C6" s="17"/>
       <c r="H6" s="2"/>
-      <c r="I6" s="22"/>
+      <c r="I6" s="19"/>
       <c r="K6" s="2"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="22"/>
-      <c r="C7" s="19"/>
+      <c r="A7" s="19"/>
+      <c r="C7" s="17"/>
       <c r="H7" s="2"/>
-      <c r="I7" s="22"/>
+      <c r="I7" s="19"/>
       <c r="K7" s="2"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="22"/>
-      <c r="C8" s="19"/>
+      <c r="A8" s="19"/>
+      <c r="C8" s="17"/>
       <c r="H8" s="2"/>
-      <c r="I8" s="22"/>
+      <c r="I8" s="19"/>
       <c r="K8" s="2"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="22"/>
-      <c r="C9" s="19"/>
+      <c r="A9" s="19"/>
+      <c r="C9" s="17"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="22"/>
+      <c r="I9" s="19"/>
       <c r="K9" s="2"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="22"/>
-      <c r="C10" s="19"/>
+      <c r="A10" s="19"/>
+      <c r="C10" s="17"/>
       <c r="H10" s="2"/>
-      <c r="I10" s="22"/>
+      <c r="I10" s="19"/>
       <c r="K10" s="2"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" s="22"/>
-      <c r="C11" s="19"/>
+      <c r="A11" s="19"/>
+      <c r="C11" s="17"/>
       <c r="H11" s="2"/>
-      <c r="I11" s="22"/>
+      <c r="I11" s="19"/>
       <c r="K11" s="2"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" s="22"/>
-      <c r="C12" s="19"/>
+      <c r="A12" s="19"/>
+      <c r="C12" s="17"/>
       <c r="H12" s="2"/>
-      <c r="I12" s="22"/>
-      <c r="K12" s="18"/>
+      <c r="I12" s="19"/>
+      <c r="K12" s="16"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A13" s="22"/>
-      <c r="C13" s="19"/>
+      <c r="A13" s="19"/>
+      <c r="C13" s="17"/>
       <c r="H13" s="2"/>
-      <c r="I13" s="22"/>
+      <c r="I13" s="19"/>
       <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" s="22"/>
-      <c r="C14" s="19"/>
+      <c r="A14" s="19"/>
+      <c r="C14" s="17"/>
       <c r="H14" s="2"/>
-      <c r="I14" s="22"/>
+      <c r="I14" s="19"/>
       <c r="K14" s="2"/>
     </row>
   </sheetData>
@@ -5349,386 +5435,386 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
     </row>
     <row r="2" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="29" t="s">
         <v>119</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
     </row>
     <row r="3" spans="1:11" ht="34" x14ac:dyDescent="0.2">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="G3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="H3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="23" t="s">
+      <c r="J3" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="K3" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="51" x14ac:dyDescent="0.2">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="21" t="s">
+      <c r="I4" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="21" t="s">
+      <c r="J4" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="K4" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="51" x14ac:dyDescent="0.2">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="21" t="s">
+      <c r="I5" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J5" s="21" t="s">
+      <c r="J5" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="K5" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="68" x14ac:dyDescent="0.2">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G6" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="21" t="s">
+      <c r="I6" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="21" t="s">
+      <c r="J6" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="K6" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="51" x14ac:dyDescent="0.2">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="21" t="s">
+      <c r="I7" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="21" t="s">
+      <c r="J7" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="K7" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="51" x14ac:dyDescent="0.2">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="21" t="s">
+      <c r="I8" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="21" t="s">
+      <c r="J8" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="K8" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="51" x14ac:dyDescent="0.2">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I9" s="21" t="s">
+      <c r="I9" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J9" s="21" t="s">
+      <c r="J9" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="K9" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="170" x14ac:dyDescent="0.2">
-      <c r="A10" s="21" t="s">
+    <row r="10" spans="1:11" ht="204" x14ac:dyDescent="0.2">
+      <c r="A10" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="D10" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="G10" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I10" s="21" t="s">
+      <c r="I10" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J10" s="21" t="s">
+      <c r="J10" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K10" s="17" t="s">
-        <v>152</v>
+      <c r="K10" s="15" t="s">
+        <v>154</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="68" x14ac:dyDescent="0.2">
-      <c r="A11" s="21" t="s">
+    <row r="11" spans="1:11" ht="119" x14ac:dyDescent="0.2">
+      <c r="A11" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="H11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I11" s="21" t="s">
+      <c r="I11" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J11" s="21" t="s">
+      <c r="J11" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K11" s="8" t="s">
-        <v>18</v>
+      <c r="K11" s="30" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="68" x14ac:dyDescent="0.2">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="G12" s="14" t="s">
+      <c r="G12" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="H12" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I12" s="21" t="s">
+      <c r="I12" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J12" s="21" t="s">
+      <c r="J12" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="K12" s="8" t="s">
+      <c r="K12" s="7" t="s">
         <v>18</v>
       </c>
     </row>
@@ -5756,427 +5842,427 @@
     <col min="7" max="7" width="44.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="37.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" style="22"/>
+    <col min="10" max="10" width="10.83203125" style="19"/>
     <col min="11" max="11" width="31.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
     </row>
     <row r="2" spans="1:11" ht="70" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="28" t="s">
-        <v>153</v>
-      </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="30"/>
+      <c r="B2" s="24" t="s">
+        <v>152</v>
+      </c>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="26"/>
     </row>
     <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="G3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="H3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="23" t="s">
+      <c r="J3" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="K3" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="102" x14ac:dyDescent="0.2">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="21" t="s">
+      <c r="J4" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="K4" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="102" x14ac:dyDescent="0.2">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="I5" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J5" s="21" t="s">
+      <c r="J5" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="K5" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="102" x14ac:dyDescent="0.2">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G6" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="16" t="s">
+      <c r="I6" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="21" t="s">
+      <c r="J6" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="K6" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="102" x14ac:dyDescent="0.2">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="I7" s="21" t="s">
+      <c r="I7" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="J7" s="21" t="s">
+      <c r="J7" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="K7" s="14" t="s">
+      <c r="K7" s="12" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="102" x14ac:dyDescent="0.2">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="I8" s="21" t="s">
+      <c r="I8" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="J8" s="21" t="s">
+      <c r="J8" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="K8" s="14" t="s">
+      <c r="K8" s="12" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="102" x14ac:dyDescent="0.2">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="H9" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="I9" s="21" t="s">
+      <c r="I9" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="J9" s="21" t="s">
+      <c r="J9" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="K9" s="14" t="s">
+      <c r="K9" s="12" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="102" x14ac:dyDescent="0.2">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="D10" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="G10" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="H10" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="I10" s="21" t="s">
+      <c r="I10" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="J10" s="21" t="s">
+      <c r="J10" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="K10" s="14" t="s">
+      <c r="K10" s="12" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="H11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I11" s="21" t="s">
+      <c r="I11" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J11" s="21" t="s">
+      <c r="J11" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="K11" s="8" t="s">
+      <c r="K11" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="G12" s="14" t="s">
+      <c r="G12" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="H12" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I12" s="21" t="s">
+      <c r="I12" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J12" s="21" t="s">
+      <c r="J12" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="K12" s="8" t="s">
+      <c r="K12" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="102" x14ac:dyDescent="0.2">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="G13" s="14" t="s">
+      <c r="G13" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="H13" s="14" t="s">
+      <c r="H13" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="I13" s="21" t="s">
+      <c r="I13" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="J13" s="21" t="s">
+      <c r="J13" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="K13" s="14" t="s">
+      <c r="K13" s="12" t="s">
         <v>66</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update of test plan (WIP)
</commit_message>
<xml_diff>
--- a/docs/TestCases.xlsx
+++ b/docs/TestCases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arcigo/Documents/Projects/BigBankDemo/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9ECF041-D743-984B-9C0B-06E90C936E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7003029-73B3-5347-BC03-13D28E064D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{5A36BFF6-BC86-D248-B9E6-C6BC71C126C7}"/>
   </bookViews>
@@ -4821,7 +4821,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4831,18 +4843,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5199,19 +5199,19 @@
       <c r="A1" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
     </row>
     <row r="2" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
@@ -5329,17 +5329,17 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="22"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="19"/>
@@ -5438,35 +5438,35 @@
       <c r="A1" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
     </row>
     <row r="2" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
     </row>
     <row r="3" spans="1:11" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
@@ -5779,7 +5779,7 @@
       <c r="J11" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K11" s="30" t="s">
+      <c r="K11" s="23" t="s">
         <v>153</v>
       </c>
     </row>
@@ -5851,35 +5851,35 @@
       <c r="A1" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
     </row>
     <row r="2" spans="1:11" ht="70" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="28" t="s">
         <v>152</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="26"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="30"/>
     </row>
     <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
@@ -6161,7 +6161,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A11" s="13" t="s">
         <v>56</v>
       </c>

</xml_diff>

<commit_message>
Update of docs. Update of tests, and its data, and add of URL parametrised test
</commit_message>
<xml_diff>
--- a/docs/TestCases.xlsx
+++ b/docs/TestCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arcigo/Documents/Projects/BigBankDemo/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7003029-73B3-5347-BC03-13D28E064D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33C86B98-94EF-9F4E-B785-0752F7373C51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{5A36BFF6-BC86-D248-B9E6-C6BC71C126C7}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29840" windowHeight="18580" activeTab="2" xr2:uid="{5A36BFF6-BC86-D248-B9E6-C6BC71C126C7}"/>
   </bookViews>
   <sheets>
     <sheet name="UI (part 1)" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="157">
   <si>
     <t>Test Case</t>
   </si>
@@ -4492,47 +4492,87 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">If I press the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Enter</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> key after filling any of the inputs of the form, or when I use the sliders, the modal closes. Is this an expected behavior? If not, this condition from the assessment is not met: </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>«Calculator changes should not be saved until the "Jätka" button is clicked»</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>APRC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is never displayed in the UI. But, By checking the Network traces in the browser, I can see that the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>calculate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> endpoint returns the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>apr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>APRC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in the UI) property.</t>
     </r>
   </si>
   <si>
@@ -4596,6 +4636,312 @@
         <scheme val="minor"/>
       </rPr>
       <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>APRC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is never displayed in the UI. But, By checking the Network traces in the browser, I can see that the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>calculate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> endpoint returns the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>apr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>APRC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in the UI) property.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">* If I press the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Enter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> key after filling any of the inputs of the form, or when I use the sliders, the modal closes. Is this an expected behavior? If not, this condition from the assessment is not met: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>«Calculator changes should not be saved until the "Jätka" button is clicked»</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>APRC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is never displayed in the UI. But, By checking the Network traces in the browser, I can see that the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>calculate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> endpoint returns the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>apr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>APRC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in the UI) property.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>APRC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is never displayed in the UI. But, By checking the Network traces in the browser, I can see that the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>calculate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> endpoint returns the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">apr </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>APRC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in the UI)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> property.
+* I added this case just to figure out how to land to the calculator modal.</t>
     </r>
   </si>
 </sst>
@@ -5192,7 +5538,8 @@
     <col min="8" max="8" width="28.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="10.83203125" style="19"/>
-    <col min="12" max="16384" width="10.83203125" style="1"/>
+    <col min="12" max="12" width="29.83203125" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="17" x14ac:dyDescent="0.2">
@@ -5251,7 +5598,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="119" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="136" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
         <v>11</v>
       </c>
@@ -5285,11 +5632,11 @@
       <c r="K3" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="7" t="s">
-        <v>18</v>
+      <c r="L3" s="23" t="s">
+        <v>156</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="68" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="85" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
         <v>19</v>
       </c>
@@ -5323,8 +5670,8 @@
       <c r="K4" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="L4" s="7" t="s">
-        <v>18</v>
+      <c r="L4" s="23" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -5713,7 +6060,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="204" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" ht="289" x14ac:dyDescent="0.2">
       <c r="A10" s="14" t="s">
         <v>37</v>
       </c>
@@ -5748,7 +6095,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="119" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" ht="204" x14ac:dyDescent="0.2">
       <c r="A11" s="14" t="s">
         <v>40</v>
       </c>
@@ -5780,7 +6127,7 @@
         <v>17</v>
       </c>
       <c r="K11" s="23" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="68" x14ac:dyDescent="0.2">

</xml_diff>